<commit_message>
RPEF edit to align with BPM assumptions
</commit_message>
<xml_diff>
--- a/InputData/trans/RPEF/Retail Price Equivalent Factor.xlsx
+++ b/InputData/trans/RPEF/Retail Price Equivalent Factor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\trans\RPEF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\RPEF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39502BE2-C6DB-4BB4-A277-8DB7845D96C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A60FCEBE-E7D7-466E-B619-1756402D7BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -945,7 +945,7 @@
       <alignment horizontal="left"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -957,8 +957,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1499,10 +1498,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="85.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="2" max="2" width="85.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1519,27 +1518,24 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="B4" s="7" t="s">
+      <c r="B4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <v>2009</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="B6" s="7" t="s">
+      <c r="B6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="B7" s="7" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="B8" s="7"/>
     </row>
     <row r="9" spans="1:2">
       <c r="B9" s="6" t="s">
@@ -1547,33 +1543,24 @@
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="B10" s="7" t="s">
+      <c r="B10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="B11" s="8">
+      <c r="B11" s="7">
         <v>2019</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="B12" s="7" t="s">
+      <c r="B12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="B13" s="7" t="s">
+      <c r="B13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="B14" s="7"/>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="B15" s="7"/>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="B16" s="7"/>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="1" t="s">
@@ -1592,13 +1579,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AK7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="45">
+    <row r="1" spans="1:37" ht="43.5">
       <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
@@ -1651,7 +1638,7 @@
         <v>1.5</v>
       </c>
       <c r="C2" s="4">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>

</xml_diff>